<commit_message>
update ui and latest local code
</commit_message>
<xml_diff>
--- a/output/标准销量表.xlsx
+++ b/output/标准销量表.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>曲靖市宣威市联启通讯智能家居店</t>
+          <t>曲靖市宣威市联启通讯建设西路12分店</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>62T02262100196722</t>
+          <t>6UNBB26311069618</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>畅享90 Pro Max Voyager-AL00E</t>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>张必然</t>
+          <t>周然</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
@@ -523,12 +523,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>曲靖市宣威市联启通讯智能家居店</t>
+          <t>曲靖市宣威市联启通讯建设西路12分店</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>张必然</t>
+          <t>周然</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -541,56 +541,828 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市交通门文昌通讯合作店</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6UNBB26315050323</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>吴智铭</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市交通门文昌通讯合作店</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市杜鹃花雕像文昌通讯合作店</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>77UYD26309020497</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Plus Judy-AL50D</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>夏淑媛</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市杜鹃花雕像文昌通讯合作店</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>云南联启通讯有限公司</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>曲靖市宣威市联启通讯建设西路12分店</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>4ZQ9K261120065372</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>畅享90 Plus Jiaolong-AN80B-DT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>6UPBB26311018414</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>周然</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
-        <v>46114</v>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="F5" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市联启通讯建设西路12分店</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>周然</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>曲靖市沾益区联启通讯西平路店</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6UPBB26311000263</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>赵蜜</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>曲靖市沾益区联启通讯西平路店</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>赵蜜</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市建设西路联启通讯合作店</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6UNBB26306004626</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>曾艳</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市建设西路联启通讯合作店</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>曲靖宣威市文昌通讯振兴中路二楼总店</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6UNBB26319042997</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>王瑜</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>宣威市同文通讯设备有限公司</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>曲靖宣威市文昌通讯振兴中路二楼总店</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>曲靖市宣威振兴街大众通讯2分店</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>77TYD26313005200</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Plus Judy-AL50C</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>钱彩艳</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>曲靖市宣威振兴街大众通讯2分店</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>钱彩艳</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6UNBB26318004724</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6UNBB26318019565</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00D</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6UPBB26317009411</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>云南联启通讯有限公司</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>曲靖市宣威市联启通讯建设西路12分店</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>77TYD26313003956</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Plus Judy-AL50C</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>周然</t>
         </is>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="F13" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市联启通讯建设西路12分店</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>周然</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>曲靖市沾益区联启通讯西平路店</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>77TYD26309027064</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Plus Judy-AL50C</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>赵蜜</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>云南联启通讯有限公司</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>曲靖市沾益区联启通讯西平路店</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>赵蜜</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市大众通讯振兴街店</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6UPBB26311018218</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>马举川</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市大众通讯振兴街店</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>马举川</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市大众通讯振兴街店</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6UPBB26308009530</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>马举川</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>宣威市朝龙商贸有限公司</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>曲靖市宣威市大众通讯振兴街店</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>马举川</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6UPBB26308003605</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>华为畅享 90 Pro Max Chenzhen-AL00E</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>云南九机电子产品有限公司</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>云南省宣威市九机网1店</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>刘博</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>